<commit_message>
Perfektionierung Projektstrukturplan (PSP) als reine, native Excel-Tabelle ohne Bildobjekt mit 5 Saeulen und 30 Arbeitspaketen
</commit_message>
<xml_diff>
--- a/docs/01_Projektorganisation/Projektstrukturplan.xlsx
+++ b/docs/01_Projektorganisation/Projektstrukturplan.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,6 +58,12 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="001F497D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="14"/>
     </font>
@@ -66,7 +72,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -95,7 +101,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F5F9"/>
+        <fgColor rgb="00F9FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBF1F5"/>
       </patternFill>
     </fill>
     <fill>
@@ -172,7 +183,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -194,19 +205,22 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -574,45 +588,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AD38"/>
+  <dimension ref="B2:AD41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="7.5" customWidth="1" min="1" max="1"/>
-    <col width="7.5" customWidth="1" min="2" max="2"/>
-    <col width="7.5" customWidth="1" min="3" max="3"/>
-    <col width="7.5" customWidth="1" min="4" max="4"/>
-    <col width="7.5" customWidth="1" min="5" max="5"/>
-    <col width="7.5" customWidth="1" min="6" max="6"/>
-    <col width="7.5" customWidth="1" min="7" max="7"/>
-    <col width="7.5" customWidth="1" min="8" max="8"/>
-    <col width="7.5" customWidth="1" min="9" max="9"/>
-    <col width="7.5" customWidth="1" min="10" max="10"/>
-    <col width="7.5" customWidth="1" min="11" max="11"/>
-    <col width="7.5" customWidth="1" min="12" max="12"/>
-    <col width="7.5" customWidth="1" min="13" max="13"/>
-    <col width="7.5" customWidth="1" min="14" max="14"/>
-    <col width="7.5" customWidth="1" min="15" max="15"/>
-    <col width="7.5" customWidth="1" min="16" max="16"/>
-    <col width="7.5" customWidth="1" min="17" max="17"/>
-    <col width="7.5" customWidth="1" min="18" max="18"/>
-    <col width="7.5" customWidth="1" min="19" max="19"/>
-    <col width="7.5" customWidth="1" min="20" max="20"/>
-    <col width="7.5" customWidth="1" min="21" max="21"/>
-    <col width="7.5" customWidth="1" min="22" max="22"/>
-    <col width="7.5" customWidth="1" min="23" max="23"/>
-    <col width="7.5" customWidth="1" min="24" max="24"/>
-    <col width="7.5" customWidth="1" min="25" max="25"/>
-    <col width="7.5" customWidth="1" min="26" max="26"/>
-    <col width="7.5" customWidth="1" min="27" max="27"/>
-    <col width="7.5" customWidth="1" min="28" max="28"/>
-    <col width="7.5" customWidth="1" min="29" max="29"/>
-    <col width="7.5" customWidth="1" min="30" max="30"/>
-    <col width="7.5" customWidth="1" min="31" max="31"/>
-    <col width="7.5" customWidth="1" min="32" max="32"/>
-    <col width="7.5" customWidth="1" min="33" max="33"/>
-    <col width="7.5" customWidth="1" min="34" max="34"/>
+    <col width="3.2" customWidth="1" min="1" max="1"/>
+    <col width="6.4" customWidth="1" min="2" max="2"/>
+    <col width="6.4" customWidth="1" min="3" max="3"/>
+    <col width="6.4" customWidth="1" min="4" max="4"/>
+    <col width="6.4" customWidth="1" min="5" max="5"/>
+    <col width="6.4" customWidth="1" min="6" max="6"/>
+    <col width="3.2" customWidth="1" min="7" max="7"/>
+    <col width="6.4" customWidth="1" min="8" max="8"/>
+    <col width="6.4" customWidth="1" min="9" max="9"/>
+    <col width="6.4" customWidth="1" min="10" max="10"/>
+    <col width="6.4" customWidth="1" min="11" max="11"/>
+    <col width="6.4" customWidth="1" min="12" max="12"/>
+    <col width="3.2" customWidth="1" min="13" max="13"/>
+    <col width="6.4" customWidth="1" min="14" max="14"/>
+    <col width="6.4" customWidth="1" min="15" max="15"/>
+    <col width="6.4" customWidth="1" min="16" max="16"/>
+    <col width="6.4" customWidth="1" min="17" max="17"/>
+    <col width="6.4" customWidth="1" min="18" max="18"/>
+    <col width="3.2" customWidth="1" min="19" max="19"/>
+    <col width="6.4" customWidth="1" min="20" max="20"/>
+    <col width="6.4" customWidth="1" min="21" max="21"/>
+    <col width="6.4" customWidth="1" min="22" max="22"/>
+    <col width="6.4" customWidth="1" min="23" max="23"/>
+    <col width="6.4" customWidth="1" min="24" max="24"/>
+    <col width="3.2" customWidth="1" min="25" max="25"/>
+    <col width="6.4" customWidth="1" min="26" max="26"/>
+    <col width="6.4" customWidth="1" min="27" max="27"/>
+    <col width="6.4" customWidth="1" min="28" max="28"/>
+    <col width="6.4" customWidth="1" min="29" max="29"/>
+    <col width="6.4" customWidth="1" min="30" max="30"/>
+    <col width="3.2" customWidth="1" min="31" max="31"/>
+    <col width="6.4" customWidth="1" min="32" max="32"/>
+    <col width="6.4" customWidth="1" min="33" max="33"/>
+    <col width="6.4" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
+    <row r="1" ht="10" customHeight="1"/>
     <row r="2" ht="32" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -623,16 +638,17 @@
     <row r="3" ht="20" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Projekt: IT-Ausstattung Planungs- und Konstruktionsbüro | Kunde: VektorPlan GmbH | Projektleiter: Jan Kluth</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="18" customHeight="1">
+          <t>Projekt: IT-Ausstattung Planungs- und Konstruktionsbüro | Kunde: VektorPlan GmbH | Projektleiter: Jan Kluth | 5 Teilprojekte, 30 Arbeitspakete</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="10" customHeight="1"/>
+    <row r="5" ht="19" customHeight="1">
       <c r="N5" s="3" t="inlineStr">
         <is>
           <t>1.0 IT-Ausstattung VektorPlan GmbH
-(Schlüsselfertige Büro-Ausstattung)
-Projektleiter: Jan Kluth</t>
+(Schlüsselfertige Büro-Gesamtausstattung)
+Projektleitung: Jan Kluth</t>
         </is>
       </c>
       <c r="O5" s="4" t="n"/>
@@ -640,24 +656,24 @@
       <c r="Q5" s="4" t="n"/>
       <c r="R5" s="4" t="n"/>
     </row>
-    <row r="6" ht="18" customHeight="1">
+    <row r="6" ht="19" customHeight="1">
       <c r="N6" s="4" t="n"/>
       <c r="O6" s="4" t="n"/>
       <c r="P6" s="4" t="n"/>
       <c r="Q6" s="4" t="n"/>
       <c r="R6" s="4" t="n"/>
     </row>
-    <row r="7" ht="18" customHeight="1">
+    <row r="7" ht="19" customHeight="1">
       <c r="N7" s="4" t="n"/>
       <c r="O7" s="4" t="n"/>
       <c r="P7" s="4" t="n"/>
       <c r="Q7" s="4" t="n"/>
       <c r="R7" s="4" t="n"/>
     </row>
-    <row r="8" ht="12" customHeight="1">
+    <row r="8" ht="10" customHeight="1">
       <c r="P8" s="5" t="n"/>
     </row>
-    <row r="9" ht="12" customHeight="1">
+    <row r="9" ht="10" customHeight="1">
       <c r="P9" s="5" t="n"/>
     </row>
     <row r="10" ht="6" customHeight="1">
@@ -1483,12 +1499,21 @@
       <c r="AC38" s="10" t="n"/>
       <c r="AD38" s="10" t="n"/>
     </row>
+    <row r="40" ht="10" customHeight="1"/>
+    <row r="41" ht="24" customHeight="1">
+      <c r="B41" s="11" t="inlineStr">
+        <is>
+          <t>PROJEKTSTRUKTURPLAN (PSP) NACH DIN 69901  |  5 TEILPROJEKTE  |  30 ARBEITSPAKETE  |  VOLLSTÄNDIGE LIEFERUNG &amp; INBETRIEBNAHME</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="38">
+  <mergeCells count="39">
     <mergeCell ref="H24:L26"/>
     <mergeCell ref="B20:F22"/>
     <mergeCell ref="N24:R26"/>
     <mergeCell ref="N20:R22"/>
+    <mergeCell ref="B41:AD41"/>
     <mergeCell ref="B16:F18"/>
     <mergeCell ref="B32:F34"/>
     <mergeCell ref="N36:R38"/>
@@ -1545,879 +1570,879 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Arbeitspaket-Übersicht nach DIN 69901 (WBS - Work Breakdown Structure)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="25" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>PSP-Code</t>
         </is>
       </c>
-      <c r="B3" s="12" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Teilprojekt / Arbeitspaket</t>
         </is>
       </c>
-      <c r="C3" s="12" t="inlineStr">
+      <c r="C3" s="13" t="inlineStr">
         <is>
           <t>Detaillierte Beschreibung</t>
         </is>
       </c>
-      <c r="D3" s="12" t="inlineStr">
+      <c r="D3" s="13" t="inlineStr">
         <is>
           <t>Verantwortlich</t>
         </is>
       </c>
-      <c r="E3" s="12" t="inlineStr">
+      <c r="E3" s="13" t="inlineStr">
         <is>
           <t>Ergebnis / Deliverable</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>1.1 Hardware-Ausstattung (Verantwortlich: Marian Bolecke)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>1.1.1</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>12x Standard-PCs</t>
         </is>
       </c>
-      <c r="C5" s="15" t="inlineStr">
+      <c r="C5" s="16" t="inlineStr">
         <is>
           <t>Lenovo ThinkCentre M70s (SFF)</t>
         </is>
       </c>
-      <c r="D5" s="14" t="inlineStr">
+      <c r="D5" s="15" t="inlineStr">
         <is>
           <t>Marian Bolecke</t>
         </is>
       </c>
-      <c r="E5" s="15" t="inlineStr">
+      <c r="E5" s="16" t="inlineStr">
         <is>
           <t>Einsatzbereite Komponente / Dokument</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>1.1.2</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="16" t="inlineStr">
         <is>
           <t>4x CAD-Workstations</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="C6" s="16" t="inlineStr">
         <is>
           <t>Lenovo ThinkStation P3 (RTX Ada)</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="D6" s="15" t="inlineStr">
         <is>
           <t>Marian Bolecke</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr">
+      <c r="E6" s="16" t="inlineStr">
         <is>
           <t>Einsatzbereite Komponente / Dokument</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>1.1.3</t>
         </is>
       </c>
-      <c r="B7" s="15" t="inlineStr">
+      <c r="B7" s="16" t="inlineStr">
         <is>
           <t>32x Ergonomie-Monitore</t>
         </is>
       </c>
-      <c r="C7" s="15" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
         <is>
           <t>Dell UltraSharp U2724D (27'' WQHD)</t>
         </is>
       </c>
-      <c r="D7" s="14" t="inlineStr">
+      <c r="D7" s="15" t="inlineStr">
         <is>
           <t>Marian Bolecke</t>
         </is>
       </c>
-      <c r="E7" s="15" t="inlineStr">
+      <c r="E7" s="16" t="inlineStr">
         <is>
           <t>Einsatzbereite Komponente / Dokument</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>1.1.4</t>
         </is>
       </c>
-      <c r="B8" s="15" t="inlineStr">
+      <c r="B8" s="16" t="inlineStr">
         <is>
           <t>16x Eingabegeräte-Sets</t>
         </is>
       </c>
-      <c r="C8" s="15" t="inlineStr">
+      <c r="C8" s="16" t="inlineStr">
         <is>
           <t>Logitech MK650 Business (Funk AES)</t>
         </is>
       </c>
-      <c r="D8" s="14" t="inlineStr">
+      <c r="D8" s="15" t="inlineStr">
         <is>
           <t>Marian Bolecke</t>
         </is>
       </c>
-      <c r="E8" s="15" t="inlineStr">
+      <c r="E8" s="16" t="inlineStr">
         <is>
           <t>Einsatzbereite Komponente / Dokument</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>1.1.5</t>
         </is>
       </c>
-      <c r="B9" s="15" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>16x Externe SSDs</t>
         </is>
       </c>
-      <c r="C9" s="15" t="inlineStr">
+      <c r="C9" s="16" t="inlineStr">
         <is>
           <t>Samsung Portable T7 Shield 1TB</t>
         </is>
       </c>
-      <c r="D9" s="14" t="inlineStr">
+      <c r="D9" s="15" t="inlineStr">
         <is>
           <t>Marian Bolecke</t>
         </is>
       </c>
-      <c r="E9" s="15" t="inlineStr">
+      <c r="E9" s="16" t="inlineStr">
         <is>
           <t>Einsatzbereite Komponente / Dokument</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="14" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>1.1.6</t>
         </is>
       </c>
-      <c r="B10" s="15" t="inlineStr">
+      <c r="B10" s="16" t="inlineStr">
         <is>
           <t>1x Farblaser-MFP</t>
         </is>
       </c>
-      <c r="C10" s="15" t="inlineStr">
+      <c r="C10" s="16" t="inlineStr">
         <is>
           <t>Lexmark CX930dse A3/A4 Drucker</t>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr">
+      <c r="D10" s="15" t="inlineStr">
         <is>
           <t>Marian Bolecke</t>
         </is>
       </c>
-      <c r="E10" s="15" t="inlineStr">
+      <c r="E10" s="16" t="inlineStr">
         <is>
           <t>Einsatzbereite Komponente / Dokument</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>1.2 Software &amp; Lizenzen (Verantwortlich: Mathias Vonau)</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="14" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>1.2.1</t>
         </is>
       </c>
-      <c r="B12" s="15" t="inlineStr">
+      <c r="B12" s="16" t="inlineStr">
         <is>
           <t>16x Windows 11 Pro</t>
         </is>
       </c>
-      <c r="C12" s="15" t="inlineStr">
+      <c r="C12" s="16" t="inlineStr">
         <is>
           <t>OEM-Lizenzen 64-Bit</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
+      <c r="D12" s="15" t="inlineStr">
         <is>
           <t>Mathias Vonau</t>
         </is>
       </c>
-      <c r="E12" s="15" t="inlineStr">
+      <c r="E12" s="16" t="inlineStr">
         <is>
           <t>Einsatzbereite Komponente / Dokument</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="14" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>1.2.2</t>
         </is>
       </c>
-      <c r="B13" s="15" t="inlineStr">
+      <c r="B13" s="16" t="inlineStr">
         <is>
           <t>16x M365 Business</t>
         </is>
       </c>
-      <c r="C13" s="15" t="inlineStr">
+      <c r="C13" s="16" t="inlineStr">
         <is>
           <t>Office Standard Jahresabos</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
+      <c r="D13" s="15" t="inlineStr">
         <is>
           <t>Mathias Vonau</t>
         </is>
       </c>
-      <c r="E13" s="15" t="inlineStr">
+      <c r="E13" s="16" t="inlineStr">
         <is>
           <t>Einsatzbereite Komponente / Dokument</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="14" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>1.2.3</t>
         </is>
       </c>
-      <c r="B14" s="15" t="inlineStr">
+      <c r="B14" s="16" t="inlineStr">
         <is>
           <t>16x Adobe Acrobat Pro</t>
         </is>
       </c>
-      <c r="C14" s="15" t="inlineStr">
+      <c r="C14" s="16" t="inlineStr">
         <is>
           <t>PDF-Prüfung &amp; digitale Signatur</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
+      <c r="D14" s="15" t="inlineStr">
         <is>
           <t>Mathias Vonau</t>
         </is>
       </c>
-      <c r="E14" s="15" t="inlineStr">
+      <c r="E14" s="16" t="inlineStr">
         <is>
           <t>Einsatzbereite Komponente / Dokument</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="14" t="inlineStr">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>1.2.4</t>
         </is>
       </c>
-      <c r="B15" s="15" t="inlineStr">
+      <c r="B15" s="16" t="inlineStr">
         <is>
           <t>16x ESET PROTECT</t>
         </is>
       </c>
-      <c r="C15" s="15" t="inlineStr">
+      <c r="C15" s="16" t="inlineStr">
         <is>
           <t>Cloud EDR Endpoint Security</t>
         </is>
       </c>
-      <c r="D15" s="14" t="inlineStr">
+      <c r="D15" s="15" t="inlineStr">
         <is>
           <t>Mathias Vonau</t>
         </is>
       </c>
-      <c r="E15" s="15" t="inlineStr">
+      <c r="E15" s="16" t="inlineStr">
         <is>
           <t>Einsatzbereite Komponente / Dokument</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="14" t="inlineStr">
+      <c r="A16" s="15" t="inlineStr">
         <is>
           <t>1.2.5</t>
         </is>
       </c>
-      <c r="B16" s="15" t="inlineStr">
+      <c r="B16" s="16" t="inlineStr">
         <is>
           <t>Software-Images</t>
         </is>
       </c>
-      <c r="C16" s="15" t="inlineStr">
+      <c r="C16" s="16" t="inlineStr">
         <is>
           <t>Vorinstallation &amp; Staging-Image</t>
         </is>
       </c>
-      <c r="D16" s="14" t="inlineStr">
+      <c r="D16" s="15" t="inlineStr">
         <is>
           <t>Mathias Vonau</t>
         </is>
       </c>
-      <c r="E16" s="15" t="inlineStr">
+      <c r="E16" s="16" t="inlineStr">
         <is>
           <t>Einsatzbereite Komponente / Dokument</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="14" t="inlineStr">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>1.2.6</t>
         </is>
       </c>
-      <c r="B17" s="15" t="inlineStr">
+      <c r="B17" s="16" t="inlineStr">
         <is>
           <t>Lizenzdokumentation</t>
         </is>
       </c>
-      <c r="C17" s="15" t="inlineStr">
+      <c r="C17" s="16" t="inlineStr">
         <is>
           <t>Nachweis- &amp; Lizenzübersicht</t>
         </is>
       </c>
-      <c r="D17" s="14" t="inlineStr">
+      <c r="D17" s="15" t="inlineStr">
         <is>
           <t>Mathias Vonau</t>
         </is>
       </c>
-      <c r="E17" s="15" t="inlineStr">
+      <c r="E17" s="16" t="inlineStr">
         <is>
           <t>Einsatzbereite Komponente / Dokument</t>
         </is>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="13" t="inlineStr">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>1.3 Netzwerk &amp; Server (Verantwortlich: Siyar)</t>
         </is>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="14" t="inlineStr">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>1.3.1</t>
         </is>
       </c>
-      <c r="B19" s="15" t="inlineStr">
+      <c r="B19" s="16" t="inlineStr">
         <is>
           <t>Gigabit Verkabelung</t>
         </is>
       </c>
-      <c r="C19" s="15" t="inlineStr">
+      <c r="C19" s="16" t="inlineStr">
         <is>
           <t>16x InLine Cat.6A Patchkabel</t>
         </is>
       </c>
-      <c r="D19" s="14" t="inlineStr">
+      <c r="D19" s="15" t="inlineStr">
         <is>
           <t>Siyar</t>
         </is>
       </c>
-      <c r="E19" s="15" t="inlineStr">
+      <c r="E19" s="16" t="inlineStr">
         <is>
           <t>Einsatzbereite Komponente / Dokument</t>
         </is>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="14" t="inlineStr">
+      <c r="A20" s="15" t="inlineStr">
         <is>
           <t>1.3.2</t>
         </is>
       </c>
-      <c r="B20" s="15" t="inlineStr">
+      <c r="B20" s="16" t="inlineStr">
         <is>
           <t>Fileserver-Kapazität</t>
         </is>
       </c>
-      <c r="C20" s="15" t="inlineStr">
+      <c r="C20" s="16" t="inlineStr">
         <is>
           <t>445 GiB Speicherbedarf (Q1)</t>
         </is>
       </c>
-      <c r="D20" s="14" t="inlineStr">
+      <c r="D20" s="15" t="inlineStr">
         <is>
           <t>Siyar</t>
         </is>
       </c>
-      <c r="E20" s="15" t="inlineStr">
+      <c r="E20" s="16" t="inlineStr">
         <is>
           <t>Einsatzbereite Komponente / Dokument</t>
         </is>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="14" t="inlineStr">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>1.3.3</t>
         </is>
       </c>
-      <c r="B21" s="15" t="inlineStr">
+      <c r="B21" s="16" t="inlineStr">
         <is>
           <t>Energiekosten-Analyse</t>
         </is>
       </c>
-      <c r="C21" s="15" t="inlineStr">
+      <c r="C21" s="16" t="inlineStr">
         <is>
           <t>1.771,26 € jährliche Stromkosten</t>
         </is>
       </c>
-      <c r="D21" s="14" t="inlineStr">
+      <c r="D21" s="15" t="inlineStr">
         <is>
           <t>Siyar</t>
         </is>
       </c>
-      <c r="E21" s="15" t="inlineStr">
+      <c r="E21" s="16" t="inlineStr">
         <is>
           <t>Einsatzbereite Komponente / Dokument</t>
         </is>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="14" t="inlineStr">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t>1.3.4</t>
         </is>
       </c>
-      <c r="B22" s="15" t="inlineStr">
+      <c r="B22" s="16" t="inlineStr">
         <is>
           <t>Switchport-Belegung</t>
         </is>
       </c>
-      <c r="C22" s="15" t="inlineStr">
+      <c r="C22" s="16" t="inlineStr">
         <is>
           <t>Zuordnung Ports 1 bis 16</t>
         </is>
       </c>
-      <c r="D22" s="14" t="inlineStr">
+      <c r="D22" s="15" t="inlineStr">
         <is>
           <t>Siyar</t>
         </is>
       </c>
-      <c r="E22" s="15" t="inlineStr">
+      <c r="E22" s="16" t="inlineStr">
         <is>
           <t>Einsatzbereite Komponente / Dokument</t>
         </is>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="14" t="inlineStr">
+      <c r="A23" s="15" t="inlineStr">
         <is>
           <t>1.3.5</t>
         </is>
       </c>
-      <c r="B23" s="15" t="inlineStr">
+      <c r="B23" s="16" t="inlineStr">
         <is>
           <t>Server-Synchronisation</t>
         </is>
       </c>
-      <c r="C23" s="15" t="inlineStr">
+      <c r="C23" s="16" t="inlineStr">
         <is>
           <t>Tägliche Sicherung der lokalen SSDs</t>
         </is>
       </c>
-      <c r="D23" s="14" t="inlineStr">
+      <c r="D23" s="15" t="inlineStr">
         <is>
           <t>Siyar</t>
         </is>
       </c>
-      <c r="E23" s="15" t="inlineStr">
+      <c r="E23" s="16" t="inlineStr">
         <is>
           <t>Einsatzbereite Komponente / Dokument</t>
         </is>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="14" t="inlineStr">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t>1.3.6</t>
         </is>
       </c>
-      <c r="B24" s="15" t="inlineStr">
+      <c r="B24" s="16" t="inlineStr">
         <is>
           <t>Netzlaufwerke &amp; Rechte</t>
         </is>
       </c>
-      <c r="C24" s="15" t="inlineStr">
+      <c r="C24" s="16" t="inlineStr">
         <is>
           <t>Konfiguration der Freigaben</t>
         </is>
       </c>
-      <c r="D24" s="14" t="inlineStr">
+      <c r="D24" s="15" t="inlineStr">
         <is>
           <t>Siyar</t>
         </is>
       </c>
-      <c r="E24" s="15" t="inlineStr">
+      <c r="E24" s="16" t="inlineStr">
         <is>
           <t>Einsatzbereite Komponente / Dokument</t>
         </is>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
-      <c r="A25" s="13" t="inlineStr">
+      <c r="A25" s="14" t="inlineStr">
         <is>
           <t>1.4 QM &amp; Logistik (Verantwortlich: Marco Schmidt)</t>
         </is>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="14" t="inlineStr">
+      <c r="A26" s="15" t="inlineStr">
         <is>
           <t>1.4.1</t>
         </is>
       </c>
-      <c r="B26" s="15" t="inlineStr">
+      <c r="B26" s="16" t="inlineStr">
         <is>
           <t>Wareneingangsprüfung</t>
         </is>
       </c>
-      <c r="C26" s="15" t="inlineStr">
+      <c r="C26" s="16" t="inlineStr">
         <is>
           <t>Prüfung gem. § 377 HGB</t>
         </is>
       </c>
-      <c r="D26" s="14" t="inlineStr">
+      <c r="D26" s="15" t="inlineStr">
         <is>
           <t>Marco Schmidt</t>
         </is>
       </c>
-      <c r="E26" s="15" t="inlineStr">
+      <c r="E26" s="16" t="inlineStr">
         <is>
           <t>Einsatzbereite Komponente / Dokument</t>
         </is>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="14" t="inlineStr">
+      <c r="A27" s="15" t="inlineStr">
         <is>
           <t>1.4.2</t>
         </is>
       </c>
-      <c r="B27" s="15" t="inlineStr">
+      <c r="B27" s="16" t="inlineStr">
         <is>
           <t>Mängelrüge Distributor</t>
         </is>
       </c>
-      <c r="C27" s="15" t="inlineStr">
+      <c r="C27" s="16" t="inlineStr">
         <is>
           <t>Fristsetzung (Gehäuse &amp; Monitor)</t>
         </is>
       </c>
-      <c r="D27" s="14" t="inlineStr">
+      <c r="D27" s="15" t="inlineStr">
         <is>
           <t>Marco Schmidt</t>
         </is>
       </c>
-      <c r="E27" s="15" t="inlineStr">
+      <c r="E27" s="16" t="inlineStr">
         <is>
           <t>Einsatzbereite Komponente / Dokument</t>
         </is>
       </c>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="14" t="inlineStr">
+      <c r="A28" s="15" t="inlineStr">
         <is>
           <t>1.4.3</t>
         </is>
       </c>
-      <c r="B28" s="15" t="inlineStr">
+      <c r="B28" s="16" t="inlineStr">
         <is>
           <t>Altdrucker-Entsorgung</t>
         </is>
       </c>
-      <c r="C28" s="15" t="inlineStr">
+      <c r="C28" s="16" t="inlineStr">
         <is>
           <t>Fachgerecht nach ElektroG/WEEE</t>
         </is>
       </c>
-      <c r="D28" s="14" t="inlineStr">
+      <c r="D28" s="15" t="inlineStr">
         <is>
           <t>Marco Schmidt</t>
         </is>
       </c>
-      <c r="E28" s="15" t="inlineStr">
+      <c r="E28" s="16" t="inlineStr">
         <is>
           <t>Einsatzbereite Komponente / Dokument</t>
         </is>
       </c>
     </row>
     <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="14" t="inlineStr">
+      <c r="A29" s="15" t="inlineStr">
         <is>
           <t>1.4.4</t>
         </is>
       </c>
-      <c r="B29" s="15" t="inlineStr">
+      <c r="B29" s="16" t="inlineStr">
         <is>
           <t>Datenschutz &amp; BSI</t>
         </is>
       </c>
-      <c r="C29" s="15" t="inlineStr">
+      <c r="C29" s="16" t="inlineStr">
         <is>
           <t>Sichere 3-fache Festplattenlöschung</t>
         </is>
       </c>
-      <c r="D29" s="14" t="inlineStr">
+      <c r="D29" s="15" t="inlineStr">
         <is>
           <t>Marco Schmidt</t>
         </is>
       </c>
-      <c r="E29" s="15" t="inlineStr">
+      <c r="E29" s="16" t="inlineStr">
         <is>
           <t>Einsatzbereite Komponente / Dokument</t>
         </is>
       </c>
     </row>
     <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="14" t="inlineStr">
+      <c r="A30" s="15" t="inlineStr">
         <is>
           <t>1.4.5</t>
         </is>
       </c>
-      <c r="B30" s="15" t="inlineStr">
+      <c r="B30" s="16" t="inlineStr">
         <is>
           <t>Entsorgungsnachweis</t>
         </is>
       </c>
-      <c r="C30" s="15" t="inlineStr">
+      <c r="C30" s="16" t="inlineStr">
         <is>
           <t>Zertifikat für VektorPlan GmbH</t>
         </is>
       </c>
-      <c r="D30" s="14" t="inlineStr">
+      <c r="D30" s="15" t="inlineStr">
         <is>
           <t>Marco Schmidt</t>
         </is>
       </c>
-      <c r="E30" s="15" t="inlineStr">
+      <c r="E30" s="16" t="inlineStr">
         <is>
           <t>Einsatzbereite Komponente / Dokument</t>
         </is>
       </c>
     </row>
     <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="14" t="inlineStr">
+      <c r="A31" s="15" t="inlineStr">
         <is>
           <t>1.4.6</t>
         </is>
       </c>
-      <c r="B31" s="15" t="inlineStr">
+      <c r="B31" s="16" t="inlineStr">
         <is>
           <t>RMA-Abwicklung</t>
         </is>
       </c>
-      <c r="C31" s="15" t="inlineStr">
+      <c r="C31" s="16" t="inlineStr">
         <is>
           <t>Nachlieferung der Tauschgeräte</t>
         </is>
       </c>
-      <c r="D31" s="14" t="inlineStr">
+      <c r="D31" s="15" t="inlineStr">
         <is>
           <t>Marco Schmidt</t>
         </is>
       </c>
-      <c r="E31" s="15" t="inlineStr">
+      <c r="E31" s="16" t="inlineStr">
         <is>
           <t>Einsatzbereite Komponente / Dokument</t>
         </is>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
-      <c r="A32" s="13" t="inlineStr">
+      <c r="A32" s="14" t="inlineStr">
         <is>
           <t>1.5 Rollout &amp; Übergabe (Verantwortlich: Jan Kluth)</t>
         </is>
       </c>
     </row>
     <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="14" t="inlineStr">
+      <c r="A33" s="15" t="inlineStr">
         <is>
           <t>1.5.1</t>
         </is>
       </c>
-      <c r="B33" s="15" t="inlineStr">
+      <c r="B33" s="16" t="inlineStr">
         <is>
           <t>Staging im Systemhaus</t>
         </is>
       </c>
-      <c r="C33" s="15" t="inlineStr">
+      <c r="C33" s="16" t="inlineStr">
         <is>
           <t>Vorinstallation im IT-Labor</t>
         </is>
       </c>
-      <c r="D33" s="14" t="inlineStr">
+      <c r="D33" s="15" t="inlineStr">
         <is>
           <t>Jan Kluth</t>
         </is>
       </c>
-      <c r="E33" s="15" t="inlineStr">
+      <c r="E33" s="16" t="inlineStr">
         <is>
           <t>Einsatzbereite Komponente / Dokument</t>
         </is>
       </c>
     </row>
     <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="14" t="inlineStr">
+      <c r="A34" s="15" t="inlineStr">
         <is>
           <t>1.5.2</t>
         </is>
       </c>
-      <c r="B34" s="15" t="inlineStr">
+      <c r="B34" s="16" t="inlineStr">
         <is>
           <t>Montage vor Ort</t>
         </is>
       </c>
-      <c r="C34" s="15" t="inlineStr">
+      <c r="C34" s="16" t="inlineStr">
         <is>
           <t>Ergonomie gem. ArbStättV</t>
         </is>
       </c>
-      <c r="D34" s="14" t="inlineStr">
+      <c r="D34" s="15" t="inlineStr">
         <is>
           <t>Jan Kluth</t>
         </is>
       </c>
-      <c r="E34" s="15" t="inlineStr">
+      <c r="E34" s="16" t="inlineStr">
         <is>
           <t>Einsatzbereite Komponente / Dokument</t>
         </is>
       </c>
     </row>
     <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="14" t="inlineStr">
+      <c r="A35" s="15" t="inlineStr">
         <is>
           <t>1.5.3</t>
         </is>
       </c>
-      <c r="B35" s="15" t="inlineStr">
+      <c r="B35" s="16" t="inlineStr">
         <is>
           <t>Funktionstests</t>
         </is>
       </c>
-      <c r="C35" s="15" t="inlineStr">
+      <c r="C35" s="16" t="inlineStr">
         <is>
           <t>Netzwerk, CAD &amp; Druckertest</t>
         </is>
       </c>
-      <c r="D35" s="14" t="inlineStr">
+      <c r="D35" s="15" t="inlineStr">
         <is>
           <t>Jan Kluth</t>
         </is>
       </c>
-      <c r="E35" s="15" t="inlineStr">
+      <c r="E35" s="16" t="inlineStr">
         <is>
           <t>Einsatzbereite Komponente / Dokument</t>
         </is>
       </c>
     </row>
     <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="14" t="inlineStr">
+      <c r="A36" s="15" t="inlineStr">
         <is>
           <t>1.5.4</t>
         </is>
       </c>
-      <c r="B36" s="15" t="inlineStr">
+      <c r="B36" s="16" t="inlineStr">
         <is>
           <t>Abnahmeprotokoll</t>
         </is>
       </c>
-      <c r="C36" s="15" t="inlineStr">
+      <c r="C36" s="16" t="inlineStr">
         <is>
           <t>Rechtskonforme Unterzeichnung</t>
         </is>
       </c>
-      <c r="D36" s="14" t="inlineStr">
+      <c r="D36" s="15" t="inlineStr">
         <is>
           <t>Jan Kluth</t>
         </is>
       </c>
-      <c r="E36" s="15" t="inlineStr">
+      <c r="E36" s="16" t="inlineStr">
         <is>
           <t>Einsatzbereite Komponente / Dokument</t>
         </is>
       </c>
     </row>
     <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="14" t="inlineStr">
+      <c r="A37" s="15" t="inlineStr">
         <is>
           <t>1.5.5</t>
         </is>
       </c>
-      <c r="B37" s="15" t="inlineStr">
+      <c r="B37" s="16" t="inlineStr">
         <is>
           <t>Projektcontrolling</t>
         </is>
       </c>
-      <c r="C37" s="15" t="inlineStr">
+      <c r="C37" s="16" t="inlineStr">
         <is>
           <t>Soll-Ist: 46 Tage / im Budget</t>
         </is>
       </c>
-      <c r="D37" s="14" t="inlineStr">
+      <c r="D37" s="15" t="inlineStr">
         <is>
           <t>Jan Kluth</t>
         </is>
       </c>
-      <c r="E37" s="15" t="inlineStr">
+      <c r="E37" s="16" t="inlineStr">
         <is>
           <t>Einsatzbereite Komponente / Dokument</t>
         </is>
       </c>
     </row>
     <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="14" t="inlineStr">
+      <c r="A38" s="15" t="inlineStr">
         <is>
           <t>1.5.6</t>
         </is>
       </c>
-      <c r="B38" s="15" t="inlineStr">
+      <c r="B38" s="16" t="inlineStr">
         <is>
           <t>Lessons Learned</t>
         </is>
       </c>
-      <c r="C38" s="15" t="inlineStr">
+      <c r="C38" s="16" t="inlineStr">
         <is>
           <t>Abschlusspräsentation vor Kunde</t>
         </is>
       </c>
-      <c r="D38" s="14" t="inlineStr">
+      <c r="D38" s="15" t="inlineStr">
         <is>
           <t>Jan Kluth</t>
         </is>
       </c>
-      <c r="E38" s="15" t="inlineStr">
+      <c r="E38" s="16" t="inlineStr">
         <is>
           <t>Einsatzbereite Komponente / Dokument</t>
         </is>

</xml_diff>